<commit_message>
Point LCOS BlockSensors and occupancy notes at the swapped EH-1/EH-3 detectors.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/wiring/LCOS_Layout_Inventory_v85.xlsx
+++ b/docs/wiring/LCOS_Layout_Inventory_v85.xlsx
@@ -28906,7 +28906,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>EH-1</t>
+          <t>EH-3</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -28996,7 +28996,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>EH-3</t>
+          <t>EH-1</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">

</xml_diff>